<commit_message>
README and other analisys
</commit_message>
<xml_diff>
--- a/Excel_Tables_xlsx/Dim_Cidade.xlsx
+++ b/Excel_Tables_xlsx/Dim_Cidade.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,16 @@
           <t>PIB_PerCapita</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Classificaçao_popula</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>PIB_Classificacao</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -485,6 +495,16 @@
       <c r="F2" t="n">
         <v>3328900</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -511,6 +531,16 @@
       <c r="F3" t="n">
         <v>4106200</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Very Big</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -537,6 +567,16 @@
       <c r="F4" t="n">
         <v>11445800</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -563,6 +603,16 @@
       <c r="F5" t="n">
         <v>2839600</v>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Big</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -589,6 +639,16 @@
       <c r="F6" t="n">
         <v>5342700</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Very Big</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -615,6 +675,16 @@
       <c r="F7" t="n">
         <v>2100600</v>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -641,6 +711,16 @@
       <c r="F8" t="n">
         <v>6482300</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -667,6 +747,16 @@
       <c r="F9" t="n">
         <v>4246000</v>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Big</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -693,6 +783,16 @@
       <c r="F10" t="n">
         <v>7514200</v>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Very Big</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -718,6 +818,16 @@
       </c>
       <c r="F11" t="n">
         <v>8435200</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Big</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>